<commit_message>
chore(data): add supporting dataset files and review workbooks
</commit_message>
<xml_diff>
--- a/Ver4/testdata/エクセル/real_article_dataset 目検.xlsx
+++ b/Ver4/testdata/エクセル/real_article_dataset 目検.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9733118985f6bf19/Desktop/datamix/講義/05_インテグレーションステップ/fake-news-checker/Ver3/testdata/エクセル/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oneuk\OneDrive\Desktop\datamix\講義\05_インテグレーションステップ\fake-news-checker\Ver4\testdata\エクセル\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{83B0F76D-0BE9-4E9E-B8AE-01038F6DD086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C221F19-AF8E-4D9E-8EF9-932BD70494CE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5449D1BB-878B-4B03-9966-4742044FFC21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{767A8689-D91E-4E19-9B42-81D7AE26A9A3}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="real_article_dataset" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">real_article_dataset!$A$1:$N$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">real_article_dataset!$A$1:$N$101</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="617">
   <si>
     <t>id</t>
   </si>
@@ -2403,6 +2403,10 @@
   </si>
   <si>
     <t>positive-accurate-14-post-23899</t>
+    <phoneticPr fontId="18"/>
+  </si>
+  <si>
+    <t>https://www.snopes.com/fact-check/biden-bounty-maduro/</t>
     <phoneticPr fontId="18"/>
   </si>
 </sst>
@@ -3418,7 +3422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2038D1B-0BDF-4C41-81D3-AA444C04F44C}">
-  <dimension ref="A1:N102"/>
+  <dimension ref="A1:N101"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="8" max="8" width="42.8984375" customWidth="1"/>
@@ -4082,39 +4086,79 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="B16" s="1"/>
-      <c r="D16" s="2"/>
+      <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E16" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>518</v>
+      </c>
+      <c r="I16" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" t="s">
+        <v>61</v>
+      </c>
+      <c r="K16" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" t="b">
+        <v>1</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>82</v>
+      </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C17" t="s">
         <v>60</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E17" t="s">
         <v>62</v>
       </c>
       <c r="F17" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G17" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="3" t="s">
-        <v>518</v>
+      <c r="H17" t="s">
+        <v>482</v>
       </c>
       <c r="I17" t="s">
         <v>19</v>
       </c>
       <c r="J17" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="K17" t="b">
         <v>1</v>
@@ -4131,34 +4175,34 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
         <v>60</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="E18" t="s">
         <v>62</v>
       </c>
       <c r="F18" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="G18" t="s">
         <v>18</v>
       </c>
       <c r="H18" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="I18" t="s">
         <v>19</v>
       </c>
       <c r="J18" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="K18" t="b">
         <v>1</v>
@@ -4175,34 +4219,34 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C19" t="s">
         <v>60</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E19" t="s">
         <v>62</v>
       </c>
       <c r="F19" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G19" t="s">
         <v>18</v>
       </c>
       <c r="H19" t="s">
-        <v>483</v>
+        <v>533</v>
       </c>
       <c r="I19" t="s">
         <v>19</v>
       </c>
       <c r="J19" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="K19" t="b">
         <v>1</v>
@@ -4219,34 +4263,34 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C20" t="s">
         <v>60</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E20" t="s">
         <v>62</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G20" t="s">
         <v>18</v>
       </c>
       <c r="H20" t="s">
-        <v>533</v>
+        <v>484</v>
       </c>
       <c r="I20" t="s">
         <v>19</v>
       </c>
       <c r="J20" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="K20" t="b">
         <v>1</v>
@@ -4263,34 +4307,34 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
         <v>60</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E21" t="s">
         <v>62</v>
       </c>
       <c r="F21" t="s">
-        <v>79</v>
+        <v>485</v>
       </c>
       <c r="G21" t="s">
         <v>18</v>
       </c>
       <c r="H21" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="I21" t="s">
         <v>19</v>
       </c>
       <c r="J21" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="K21" t="b">
         <v>1</v>
@@ -4307,34 +4351,34 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>81</v>
+        <v>499</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E22" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="F22" t="s">
-        <v>485</v>
+        <v>491</v>
       </c>
       <c r="G22" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="H22" t="s">
-        <v>486</v>
+        <v>500</v>
       </c>
       <c r="I22" t="s">
         <v>19</v>
       </c>
       <c r="J22" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="K22" t="b">
         <v>1</v>
@@ -4351,34 +4395,34 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>499</v>
+        <v>554</v>
       </c>
       <c r="C23" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>368</v>
+        <v>552</v>
       </c>
       <c r="E23" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="F23" t="s">
-        <v>491</v>
+        <v>555</v>
       </c>
       <c r="G23" t="s">
         <v>85</v>
       </c>
       <c r="H23" t="s">
-        <v>500</v>
+        <v>553</v>
       </c>
       <c r="I23" t="s">
         <v>19</v>
       </c>
       <c r="J23" t="s">
-        <v>84</v>
+        <v>552</v>
       </c>
       <c r="K23" t="b">
         <v>1</v>
@@ -4395,34 +4439,34 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>554</v>
+        <v>88</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>552</v>
+        <v>369</v>
       </c>
       <c r="E24" t="s">
-        <v>62</v>
+        <v>16</v>
       </c>
       <c r="F24" t="s">
-        <v>555</v>
+        <v>90</v>
       </c>
       <c r="G24" t="s">
         <v>85</v>
       </c>
       <c r="H24" t="s">
-        <v>553</v>
+        <v>494</v>
       </c>
       <c r="I24" t="s">
         <v>19</v>
       </c>
       <c r="J24" t="s">
-        <v>552</v>
+        <v>89</v>
       </c>
       <c r="K24" t="b">
         <v>1</v>
@@ -4434,39 +4478,39 @@
         <v>1</v>
       </c>
       <c r="N24">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>88</v>
+        <v>492</v>
       </c>
       <c r="C25" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E25" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="F25" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G25" t="s">
         <v>85</v>
       </c>
       <c r="H25" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="I25" t="s">
         <v>19</v>
       </c>
       <c r="J25" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="K25" t="b">
         <v>1</v>
@@ -4475,7 +4519,7 @@
         <v>1</v>
       </c>
       <c r="M25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N25">
         <v>80</v>
@@ -4483,34 +4527,34 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>492</v>
+        <v>550</v>
       </c>
       <c r="C26" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>370</v>
+        <v>549</v>
       </c>
       <c r="E26" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="F26" t="s">
-        <v>92</v>
+        <v>551</v>
       </c>
       <c r="G26" t="s">
         <v>85</v>
       </c>
       <c r="H26" t="s">
-        <v>493</v>
+        <v>550</v>
       </c>
       <c r="I26" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J26" t="s">
-        <v>93</v>
+        <v>549</v>
       </c>
       <c r="K26" t="b">
         <v>1</v>
@@ -4519,42 +4563,42 @@
         <v>1</v>
       </c>
       <c r="M26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N26">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>550</v>
+        <v>537</v>
       </c>
       <c r="C27" t="s">
         <v>60</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>549</v>
+        <v>538</v>
       </c>
       <c r="E27" t="s">
         <v>62</v>
       </c>
       <c r="F27" t="s">
-        <v>551</v>
+        <v>539</v>
       </c>
       <c r="G27" t="s">
         <v>85</v>
       </c>
       <c r="H27" t="s">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="I27" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="J27" t="s">
-        <v>549</v>
+        <v>538</v>
       </c>
       <c r="K27" t="b">
         <v>1</v>
@@ -4571,34 +4615,34 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="C28" t="s">
         <v>60</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="E28" t="s">
         <v>62</v>
       </c>
       <c r="F28" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="G28" t="s">
         <v>85</v>
       </c>
       <c r="H28" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="I28" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J28" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="K28" t="b">
         <v>1</v>
@@ -4615,34 +4659,34 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="C29" t="s">
         <v>60</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="E29" t="s">
         <v>62</v>
       </c>
       <c r="F29" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="G29" t="s">
         <v>85</v>
       </c>
       <c r="H29" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="I29" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J29" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="K29" t="b">
         <v>1</v>
@@ -4659,34 +4703,34 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>543</v>
+        <v>497</v>
       </c>
       <c r="C30" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>544</v>
+        <v>371</v>
       </c>
       <c r="E30" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="F30" t="s">
-        <v>545</v>
+        <v>99</v>
       </c>
       <c r="G30" t="s">
         <v>85</v>
       </c>
       <c r="H30" t="s">
-        <v>548</v>
+        <v>498</v>
       </c>
       <c r="I30" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J30" t="s">
-        <v>544</v>
+        <v>100</v>
       </c>
       <c r="K30" t="b">
         <v>1</v>
@@ -4695,42 +4739,42 @@
         <v>1</v>
       </c>
       <c r="M30">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N30">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="C31" t="s">
         <v>37</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E31" t="s">
         <v>38</v>
       </c>
       <c r="F31" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="G31" t="s">
         <v>85</v>
       </c>
       <c r="H31" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="I31" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="J31" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="K31" t="b">
         <v>1</v>
@@ -4747,34 +4791,34 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="C32" t="s">
         <v>37</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E32" t="s">
         <v>38</v>
       </c>
       <c r="F32" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="G32" t="s">
         <v>85</v>
       </c>
       <c r="H32" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="I32" t="s">
         <v>42</v>
       </c>
       <c r="J32" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="K32" t="b">
         <v>1</v>
@@ -4791,34 +4835,34 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="C33" t="s">
         <v>37</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E33" t="s">
         <v>38</v>
       </c>
       <c r="F33" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="G33" t="s">
         <v>85</v>
       </c>
       <c r="H33" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="I33" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J33" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="K33" t="b">
         <v>1</v>
@@ -4835,34 +4879,34 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>505</v>
+        <v>111</v>
       </c>
       <c r="C34" t="s">
         <v>37</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E34" t="s">
         <v>38</v>
       </c>
       <c r="F34" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="G34" t="s">
         <v>85</v>
       </c>
       <c r="H34" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="I34" t="s">
         <v>19</v>
       </c>
       <c r="J34" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="K34" t="b">
         <v>1</v>
@@ -4879,34 +4923,34 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C35" t="s">
-        <v>37</v>
+        <v>116</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E35" t="s">
-        <v>38</v>
+        <v>117</v>
       </c>
       <c r="F35" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="G35" t="s">
         <v>85</v>
       </c>
       <c r="H35" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="I35" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J35" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="K35" t="b">
         <v>1</v>
@@ -4918,39 +4962,39 @@
         <v>2</v>
       </c>
       <c r="N35">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C36" t="s">
-        <v>116</v>
+        <v>37</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E36" t="s">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="F36" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="G36" t="s">
         <v>85</v>
       </c>
       <c r="H36" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="I36" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J36" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="K36" t="b">
         <v>1</v>
@@ -4959,7 +5003,7 @@
         <v>1</v>
       </c>
       <c r="M36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N36">
         <v>82</v>
@@ -4967,34 +5011,34 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C37" t="s">
         <v>37</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E37" t="s">
         <v>57</v>
       </c>
       <c r="F37" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="G37" t="s">
         <v>85</v>
       </c>
       <c r="H37" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="I37" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J37" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="K37" t="b">
         <v>1</v>
@@ -5011,34 +5055,34 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C38" t="s">
         <v>37</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E38" t="s">
         <v>57</v>
       </c>
       <c r="F38" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="G38" t="s">
         <v>85</v>
       </c>
       <c r="H38" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="I38" t="s">
         <v>33</v>
       </c>
       <c r="J38" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="K38" t="b">
         <v>1</v>
@@ -5050,39 +5094,39 @@
         <v>1</v>
       </c>
       <c r="N38">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C39" t="s">
-        <v>37</v>
+        <v>134</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E39" t="s">
-        <v>57</v>
+        <v>136</v>
       </c>
       <c r="F39" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="G39" t="s">
         <v>85</v>
       </c>
       <c r="H39" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="I39" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="J39" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="K39" t="b">
         <v>1</v>
@@ -5094,39 +5138,39 @@
         <v>1</v>
       </c>
       <c r="N39">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>133</v>
+        <v>513</v>
       </c>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>60</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E40" t="s">
-        <v>136</v>
+        <v>62</v>
       </c>
       <c r="F40" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="G40" t="s">
         <v>85</v>
       </c>
       <c r="H40" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="I40" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J40" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="K40" t="b">
         <v>1</v>
@@ -5143,34 +5187,34 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="C41" t="s">
         <v>60</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>381</v>
+        <v>616</v>
       </c>
       <c r="E41" t="s">
         <v>62</v>
       </c>
       <c r="F41" t="s">
-        <v>140</v>
+        <v>516</v>
       </c>
       <c r="G41" t="s">
         <v>85</v>
       </c>
       <c r="H41" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="I41" t="s">
-        <v>19</v>
+        <v>478</v>
       </c>
       <c r="J41" t="s">
-        <v>139</v>
+        <v>515</v>
       </c>
       <c r="K41" t="b">
         <v>1</v>
@@ -5187,34 +5231,34 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>517</v>
+        <v>143</v>
       </c>
       <c r="C42" t="s">
-        <v>60</v>
-      </c>
-      <c r="D42" t="s">
-        <v>515</v>
+        <v>14</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>382</v>
       </c>
       <c r="E42" t="s">
-        <v>62</v>
+        <v>145</v>
       </c>
       <c r="F42" t="s">
-        <v>516</v>
+        <v>146</v>
       </c>
       <c r="G42" t="s">
-        <v>85</v>
+        <v>147</v>
       </c>
       <c r="H42" t="s">
-        <v>517</v>
+        <v>572</v>
       </c>
       <c r="I42" t="s">
-        <v>478</v>
+        <v>19</v>
       </c>
       <c r="J42" t="s">
-        <v>515</v>
+        <v>144</v>
       </c>
       <c r="K42" t="b">
         <v>1</v>
@@ -5231,34 +5275,34 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>143</v>
+        <v>574</v>
       </c>
       <c r="C43" t="s">
         <v>14</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E43" t="s">
         <v>145</v>
       </c>
       <c r="F43" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="G43" t="s">
         <v>147</v>
       </c>
       <c r="H43" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="I43" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J43" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="K43" t="b">
         <v>1</v>
@@ -5275,34 +5319,34 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>574</v>
+        <v>152</v>
       </c>
       <c r="C44" t="s">
         <v>14</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E44" t="s">
         <v>145</v>
       </c>
       <c r="F44" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="G44" t="s">
         <v>147</v>
       </c>
       <c r="H44" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="I44" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="J44" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="K44" t="b">
         <v>1</v>
@@ -5319,34 +5363,34 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>152</v>
+        <v>576</v>
       </c>
       <c r="C45" t="s">
         <v>14</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E45" t="s">
         <v>145</v>
       </c>
       <c r="F45" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="G45" t="s">
         <v>147</v>
       </c>
       <c r="H45" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="I45" t="s">
         <v>19</v>
       </c>
       <c r="J45" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="K45" t="b">
         <v>1</v>
@@ -5363,34 +5407,34 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>576</v>
+        <v>594</v>
       </c>
       <c r="C46" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>385</v>
+        <v>605</v>
       </c>
       <c r="E46" t="s">
-        <v>145</v>
+        <v>567</v>
       </c>
       <c r="F46" t="s">
-        <v>157</v>
+        <v>596</v>
       </c>
       <c r="G46" t="s">
         <v>147</v>
       </c>
       <c r="H46" t="s">
-        <v>577</v>
+        <v>609</v>
       </c>
       <c r="I46" t="s">
         <v>19</v>
       </c>
       <c r="J46" t="s">
-        <v>156</v>
+        <v>595</v>
       </c>
       <c r="K46" t="b">
         <v>1</v>
@@ -5407,34 +5451,34 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>594</v>
+        <v>160</v>
       </c>
       <c r="C47" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>605</v>
+        <v>386</v>
       </c>
       <c r="E47" t="s">
-        <v>567</v>
+        <v>145</v>
       </c>
       <c r="F47" t="s">
-        <v>596</v>
+        <v>586</v>
       </c>
       <c r="G47" t="s">
         <v>147</v>
       </c>
       <c r="H47" t="s">
-        <v>609</v>
+        <v>587</v>
       </c>
       <c r="I47" t="s">
         <v>19</v>
       </c>
       <c r="J47" t="s">
-        <v>595</v>
+        <v>161</v>
       </c>
       <c r="K47" t="b">
         <v>1</v>
@@ -5451,34 +5495,34 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>160</v>
+        <v>588</v>
       </c>
       <c r="C48" t="s">
         <v>14</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E48" t="s">
         <v>145</v>
       </c>
       <c r="F48" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="G48" t="s">
         <v>147</v>
       </c>
       <c r="H48" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="I48" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="J48" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K48" t="b">
         <v>1</v>
@@ -5495,34 +5539,34 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>588</v>
+        <v>613</v>
       </c>
       <c r="C49" t="s">
         <v>14</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E49" t="s">
         <v>145</v>
       </c>
       <c r="F49" t="s">
-        <v>589</v>
+        <v>166</v>
       </c>
       <c r="G49" t="s">
         <v>147</v>
       </c>
       <c r="H49" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="I49" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="J49" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="K49" t="b">
         <v>1</v>
@@ -5539,34 +5583,34 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="C50" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>388</v>
+        <v>606</v>
       </c>
       <c r="E50" t="s">
-        <v>145</v>
+        <v>567</v>
       </c>
       <c r="F50" t="s">
-        <v>166</v>
+        <v>598</v>
       </c>
       <c r="G50" t="s">
         <v>147</v>
       </c>
       <c r="H50" t="s">
-        <v>590</v>
+        <v>610</v>
       </c>
       <c r="I50" t="s">
         <v>19</v>
       </c>
       <c r="J50" t="s">
-        <v>165</v>
+        <v>597</v>
       </c>
       <c r="K50" t="b">
         <v>1</v>
@@ -5583,34 +5627,34 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>614</v>
+        <v>592</v>
       </c>
       <c r="C51" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>606</v>
+        <v>389</v>
       </c>
       <c r="E51" t="s">
-        <v>567</v>
+        <v>145</v>
       </c>
       <c r="F51" t="s">
-        <v>598</v>
+        <v>170</v>
       </c>
       <c r="G51" t="s">
         <v>147</v>
       </c>
       <c r="H51" t="s">
-        <v>610</v>
+        <v>593</v>
       </c>
       <c r="I51" t="s">
         <v>19</v>
       </c>
       <c r="J51" t="s">
-        <v>597</v>
+        <v>169</v>
       </c>
       <c r="K51" t="b">
         <v>1</v>
@@ -5627,34 +5671,34 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
       <c r="C52" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>389</v>
+        <v>607</v>
       </c>
       <c r="E52" t="s">
-        <v>145</v>
+        <v>567</v>
       </c>
       <c r="F52" t="s">
-        <v>170</v>
+        <v>601</v>
       </c>
       <c r="G52" t="s">
         <v>147</v>
       </c>
       <c r="H52" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
       <c r="I52" t="s">
         <v>19</v>
       </c>
       <c r="J52" t="s">
-        <v>169</v>
+        <v>600</v>
       </c>
       <c r="K52" t="b">
         <v>1</v>
@@ -5671,34 +5715,34 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>599</v>
+        <v>173</v>
       </c>
       <c r="C53" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>607</v>
+        <v>390</v>
       </c>
       <c r="E53" t="s">
-        <v>567</v>
+        <v>145</v>
       </c>
       <c r="F53" t="s">
-        <v>601</v>
+        <v>175</v>
       </c>
       <c r="G53" t="s">
         <v>147</v>
       </c>
       <c r="H53" t="s">
-        <v>612</v>
+        <v>585</v>
       </c>
       <c r="I53" t="s">
         <v>19</v>
       </c>
       <c r="J53" t="s">
-        <v>600</v>
+        <v>174</v>
       </c>
       <c r="K53" t="b">
         <v>1</v>
@@ -5715,34 +5759,34 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C54" t="s">
         <v>14</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E54" t="s">
         <v>145</v>
       </c>
       <c r="F54" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="G54" t="s">
         <v>147</v>
       </c>
       <c r="H54" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="I54" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="J54" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="K54" t="b">
         <v>1</v>
@@ -5759,34 +5803,34 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C55" t="s">
         <v>14</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E55" t="s">
         <v>145</v>
       </c>
       <c r="F55" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="G55" t="s">
         <v>147</v>
       </c>
       <c r="H55" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="I55" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="J55" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="K55" t="b">
         <v>1</v>
@@ -5803,34 +5847,34 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C56" t="s">
         <v>14</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E56" t="s">
         <v>145</v>
       </c>
       <c r="F56" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="G56" t="s">
         <v>147</v>
       </c>
       <c r="H56" t="s">
-        <v>583</v>
+        <v>580</v>
       </c>
       <c r="I56" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J56" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="K56" t="b">
         <v>1</v>
@@ -5847,34 +5891,34 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C57" t="s">
         <v>14</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E57" t="s">
         <v>145</v>
       </c>
       <c r="F57" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="G57" t="s">
         <v>147</v>
       </c>
       <c r="H57" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="I57" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="J57" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="K57" t="b">
         <v>1</v>
@@ -5891,34 +5935,34 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>189</v>
+        <v>602</v>
       </c>
       <c r="C58" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>394</v>
+        <v>608</v>
       </c>
       <c r="E58" t="s">
-        <v>145</v>
+        <v>567</v>
       </c>
       <c r="F58" t="s">
-        <v>191</v>
+        <v>604</v>
       </c>
       <c r="G58" t="s">
         <v>147</v>
       </c>
       <c r="H58" t="s">
-        <v>581</v>
+        <v>611</v>
       </c>
       <c r="I58" t="s">
         <v>19</v>
       </c>
       <c r="J58" t="s">
-        <v>190</v>
+        <v>603</v>
       </c>
       <c r="K58" t="b">
         <v>1</v>
@@ -5935,34 +5979,34 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>602</v>
+        <v>194</v>
       </c>
       <c r="C59" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>608</v>
+        <v>395</v>
       </c>
       <c r="E59" t="s">
-        <v>567</v>
+        <v>145</v>
       </c>
       <c r="F59" t="s">
-        <v>604</v>
+        <v>196</v>
       </c>
       <c r="G59" t="s">
         <v>147</v>
       </c>
       <c r="H59" t="s">
-        <v>611</v>
+        <v>582</v>
       </c>
       <c r="I59" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J59" t="s">
-        <v>603</v>
+        <v>195</v>
       </c>
       <c r="K59" t="b">
         <v>1</v>
@@ -5979,34 +6023,34 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C60" t="s">
         <v>14</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E60" t="s">
         <v>145</v>
       </c>
       <c r="F60" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="G60" t="s">
         <v>147</v>
       </c>
       <c r="H60" t="s">
-        <v>582</v>
+        <v>579</v>
       </c>
       <c r="I60" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="J60" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="K60" t="b">
         <v>1</v>
@@ -6023,34 +6067,34 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C61" t="s">
         <v>14</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E61" t="s">
         <v>145</v>
       </c>
       <c r="F61" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="G61" t="s">
         <v>147</v>
       </c>
       <c r="H61" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="I61" t="s">
         <v>19</v>
       </c>
       <c r="J61" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="K61" t="b">
         <v>1</v>
@@ -6067,34 +6111,34 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C62" t="s">
         <v>14</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E62" t="s">
         <v>145</v>
       </c>
       <c r="F62" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="G62" t="s">
-        <v>147</v>
+        <v>209</v>
       </c>
       <c r="H62" t="s">
-        <v>578</v>
+        <v>465</v>
       </c>
       <c r="I62" t="s">
         <v>19</v>
       </c>
       <c r="J62" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="K62" t="b">
         <v>1</v>
@@ -6111,34 +6155,34 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C63" t="s">
         <v>14</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="E63" t="s">
         <v>145</v>
       </c>
       <c r="F63" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="G63" t="s">
         <v>209</v>
       </c>
       <c r="H63" t="s">
-        <v>465</v>
+        <v>558</v>
       </c>
       <c r="I63" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J63" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="K63" t="b">
         <v>1</v>
@@ -6155,34 +6199,34 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C64" t="s">
         <v>14</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E64" t="s">
         <v>145</v>
       </c>
       <c r="F64" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="G64" t="s">
         <v>209</v>
       </c>
-      <c r="H64" t="s">
-        <v>558</v>
+      <c r="H64" s="4" t="s">
+        <v>557</v>
       </c>
       <c r="I64" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J64" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="K64" t="b">
         <v>1</v>
@@ -6199,34 +6243,34 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="C65" t="s">
         <v>14</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E65" t="s">
         <v>145</v>
       </c>
       <c r="F65" t="s">
-        <v>217</v>
+        <v>463</v>
       </c>
       <c r="G65" t="s">
         <v>209</v>
       </c>
-      <c r="H65" s="4" t="s">
-        <v>557</v>
+      <c r="H65" t="s">
+        <v>464</v>
       </c>
       <c r="I65" t="s">
         <v>19</v>
       </c>
       <c r="J65" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="K65" t="b">
         <v>1</v>
@@ -6243,34 +6287,34 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>219</v>
+        <v>559</v>
       </c>
       <c r="C66" t="s">
         <v>14</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E66" t="s">
         <v>145</v>
       </c>
       <c r="F66" t="s">
-        <v>463</v>
+        <v>223</v>
       </c>
       <c r="G66" t="s">
         <v>209</v>
       </c>
       <c r="H66" t="s">
-        <v>464</v>
+        <v>560</v>
       </c>
       <c r="I66" t="s">
         <v>19</v>
       </c>
       <c r="J66" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="K66" t="b">
         <v>1</v>
@@ -6287,34 +6331,34 @@
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>559</v>
+        <v>225</v>
       </c>
       <c r="C67" t="s">
         <v>14</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E67" t="s">
         <v>145</v>
       </c>
       <c r="F67" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="G67" t="s">
         <v>209</v>
       </c>
       <c r="H67" t="s">
-        <v>560</v>
+        <v>462</v>
       </c>
       <c r="I67" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J67" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="K67" t="b">
         <v>1</v>
@@ -6331,34 +6375,34 @@
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>225</v>
+        <v>561</v>
       </c>
       <c r="C68" t="s">
         <v>14</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E68" t="s">
         <v>145</v>
       </c>
       <c r="F68" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G68" t="s">
         <v>209</v>
       </c>
       <c r="H68" t="s">
-        <v>462</v>
+        <v>562</v>
       </c>
       <c r="I68" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="J68" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="K68" t="b">
         <v>1</v>
@@ -6375,34 +6419,34 @@
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>561</v>
+        <v>232</v>
       </c>
       <c r="C69" t="s">
         <v>14</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E69" t="s">
         <v>145</v>
       </c>
       <c r="F69" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="G69" t="s">
         <v>209</v>
       </c>
       <c r="H69" t="s">
-        <v>562</v>
+        <v>461</v>
       </c>
       <c r="I69" t="s">
         <v>19</v>
       </c>
       <c r="J69" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="K69" t="b">
         <v>1</v>
@@ -6419,34 +6463,34 @@
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>232</v>
+        <v>563</v>
       </c>
       <c r="C70" t="s">
         <v>14</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E70" t="s">
         <v>145</v>
       </c>
       <c r="F70" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="G70" t="s">
         <v>209</v>
       </c>
       <c r="H70" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="I70" t="s">
         <v>19</v>
       </c>
       <c r="J70" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="K70" t="b">
         <v>1</v>
@@ -6463,34 +6507,34 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
       <c r="C71" t="s">
-        <v>14</v>
+        <v>60</v>
       </c>
       <c r="D71" s="2" t="s">
-        <v>406</v>
+        <v>571</v>
       </c>
       <c r="E71" t="s">
-        <v>145</v>
+        <v>567</v>
       </c>
       <c r="F71" t="s">
-        <v>237</v>
+        <v>569</v>
       </c>
       <c r="G71" t="s">
         <v>209</v>
       </c>
       <c r="H71" t="s">
-        <v>460</v>
+        <v>570</v>
       </c>
       <c r="I71" t="s">
         <v>19</v>
       </c>
       <c r="J71" t="s">
-        <v>236</v>
+        <v>568</v>
       </c>
       <c r="K71" t="b">
         <v>1</v>
@@ -6507,34 +6551,34 @@
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>570</v>
+        <v>240</v>
       </c>
       <c r="C72" t="s">
-        <v>60</v>
+        <v>14</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>571</v>
+        <v>407</v>
       </c>
       <c r="E72" t="s">
-        <v>567</v>
+        <v>145</v>
       </c>
       <c r="F72" t="s">
-        <v>569</v>
+        <v>242</v>
       </c>
       <c r="G72" t="s">
         <v>209</v>
       </c>
       <c r="H72" t="s">
-        <v>570</v>
+        <v>459</v>
       </c>
       <c r="I72" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="J72" t="s">
-        <v>568</v>
+        <v>241</v>
       </c>
       <c r="K72" t="b">
         <v>1</v>
@@ -6551,34 +6595,34 @@
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C73" t="s">
         <v>14</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E73" t="s">
         <v>145</v>
       </c>
       <c r="F73" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="G73" t="s">
         <v>209</v>
       </c>
       <c r="H73" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="I73" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="J73" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="K73" t="b">
         <v>1</v>
@@ -6595,34 +6639,34 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C74" t="s">
         <v>14</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E74" t="s">
         <v>145</v>
       </c>
       <c r="F74" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="G74" t="s">
         <v>209</v>
       </c>
       <c r="H74" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="I74" t="s">
         <v>19</v>
       </c>
       <c r="J74" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="K74" t="b">
         <v>1</v>
@@ -6639,34 +6683,34 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C75" t="s">
         <v>14</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E75" t="s">
         <v>145</v>
       </c>
       <c r="F75" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="G75" t="s">
         <v>209</v>
       </c>
       <c r="H75" t="s">
-        <v>457</v>
+        <v>564</v>
       </c>
       <c r="I75" t="s">
         <v>19</v>
       </c>
       <c r="J75" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="K75" t="b">
         <v>1</v>
@@ -6683,34 +6727,34 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="C76" t="s">
         <v>14</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E76" t="s">
         <v>145</v>
       </c>
       <c r="F76" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="G76" t="s">
         <v>209</v>
       </c>
       <c r="H76" t="s">
-        <v>564</v>
+        <v>455</v>
       </c>
       <c r="I76" t="s">
         <v>19</v>
       </c>
       <c r="J76" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="K76" t="b">
         <v>1</v>
@@ -6727,34 +6771,34 @@
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="C77" t="s">
         <v>14</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E77" t="s">
         <v>145</v>
       </c>
       <c r="F77" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="G77" t="s">
         <v>209</v>
       </c>
       <c r="H77" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I77" t="s">
         <v>19</v>
       </c>
       <c r="J77" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="K77" t="b">
         <v>1</v>
@@ -6771,34 +6815,34 @@
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C78" t="s">
         <v>14</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E78" t="s">
         <v>145</v>
       </c>
       <c r="F78" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="G78" t="s">
         <v>209</v>
       </c>
       <c r="H78" t="s">
-        <v>456</v>
+        <v>565</v>
       </c>
       <c r="I78" t="s">
         <v>19</v>
       </c>
       <c r="J78" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="K78" t="b">
         <v>1</v>
@@ -6815,34 +6859,34 @@
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C79" t="s">
         <v>14</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E79" t="s">
         <v>145</v>
       </c>
       <c r="F79" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="G79" t="s">
         <v>209</v>
       </c>
       <c r="H79" t="s">
-        <v>565</v>
+        <v>454</v>
       </c>
       <c r="I79" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J79" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="K79" t="b">
         <v>1</v>
@@ -6859,34 +6903,34 @@
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="C80" t="s">
         <v>14</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E80" t="s">
         <v>145</v>
       </c>
       <c r="F80" t="s">
-        <v>270</v>
+        <v>452</v>
       </c>
       <c r="G80" t="s">
         <v>209</v>
       </c>
       <c r="H80" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="I80" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J80" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="K80" t="b">
         <v>1</v>
@@ -6903,34 +6947,34 @@
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C81" t="s">
         <v>14</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="E81" t="s">
         <v>145</v>
       </c>
       <c r="F81" t="s">
-        <v>452</v>
+        <v>277</v>
       </c>
       <c r="G81" t="s">
         <v>209</v>
       </c>
       <c r="H81" t="s">
-        <v>453</v>
+        <v>442</v>
       </c>
       <c r="I81" t="s">
         <v>19</v>
       </c>
       <c r="J81" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="K81" t="b">
         <v>1</v>
@@ -6947,34 +6991,34 @@
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C82" t="s">
         <v>14</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E82" t="s">
         <v>145</v>
       </c>
       <c r="F82" t="s">
-        <v>277</v>
+        <v>556</v>
       </c>
       <c r="G82" t="s">
-        <v>209</v>
+        <v>281</v>
       </c>
       <c r="H82" t="s">
-        <v>442</v>
+        <v>280</v>
       </c>
       <c r="I82" t="s">
         <v>19</v>
       </c>
       <c r="J82" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="K82" t="b">
         <v>1</v>
@@ -6991,34 +7035,34 @@
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="C83" t="s">
         <v>14</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E83" t="s">
         <v>145</v>
       </c>
       <c r="F83" t="s">
-        <v>556</v>
+        <v>285</v>
       </c>
       <c r="G83" t="s">
         <v>281</v>
       </c>
       <c r="H83" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="I83" t="s">
         <v>19</v>
       </c>
       <c r="J83" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="K83" t="b">
         <v>1</v>
@@ -7035,34 +7079,34 @@
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="C84" t="s">
         <v>14</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E84" t="s">
         <v>145</v>
       </c>
       <c r="F84" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="G84" t="s">
         <v>281</v>
       </c>
       <c r="H84" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="I84" t="s">
         <v>19</v>
       </c>
       <c r="J84" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="K84" t="b">
         <v>1</v>
@@ -7079,34 +7123,34 @@
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="C85" t="s">
         <v>14</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="E85" t="s">
         <v>145</v>
       </c>
       <c r="F85" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="G85" t="s">
         <v>281</v>
       </c>
       <c r="H85" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="I85" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="J85" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="K85" t="b">
         <v>1</v>
@@ -7123,34 +7167,34 @@
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="C86" t="s">
         <v>14</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E86" t="s">
         <v>145</v>
       </c>
       <c r="F86" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="G86" t="s">
         <v>281</v>
       </c>
       <c r="H86" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="I86" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="J86" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="K86" t="b">
         <v>1</v>
@@ -7167,34 +7211,34 @@
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="C87" t="s">
         <v>14</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E87" t="s">
         <v>145</v>
       </c>
       <c r="F87" t="s">
-        <v>297</v>
+        <v>451</v>
       </c>
       <c r="G87" t="s">
         <v>281</v>
       </c>
       <c r="H87" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="I87" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="J87" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="K87" t="b">
         <v>1</v>
@@ -7211,34 +7255,34 @@
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="C88" t="s">
         <v>14</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E88" t="s">
         <v>145</v>
       </c>
       <c r="F88" t="s">
-        <v>451</v>
+        <v>305</v>
       </c>
       <c r="G88" t="s">
         <v>281</v>
       </c>
       <c r="H88" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="I88" t="s">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="J88" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="K88" t="b">
         <v>1</v>
@@ -7255,34 +7299,34 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="C89" t="s">
         <v>14</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="E89" t="s">
         <v>145</v>
       </c>
       <c r="F89" t="s">
-        <v>305</v>
+        <v>450</v>
       </c>
       <c r="G89" t="s">
         <v>281</v>
       </c>
       <c r="H89" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="I89" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="J89" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="K89" t="b">
         <v>1</v>
@@ -7299,34 +7343,34 @@
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="C90" t="s">
         <v>14</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="E90" t="s">
         <v>145</v>
       </c>
       <c r="F90" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="G90" t="s">
         <v>281</v>
       </c>
       <c r="H90" t="s">
-        <v>309</v>
+        <v>449</v>
       </c>
       <c r="I90" t="s">
         <v>19</v>
       </c>
       <c r="J90" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="K90" t="b">
         <v>1</v>
@@ -7343,34 +7387,34 @@
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C91" t="s">
         <v>14</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E91" t="s">
         <v>145</v>
       </c>
       <c r="F91" t="s">
-        <v>449</v>
+        <v>316</v>
       </c>
       <c r="G91" t="s">
         <v>281</v>
       </c>
       <c r="H91" t="s">
-        <v>449</v>
+        <v>316</v>
       </c>
       <c r="I91" t="s">
         <v>19</v>
       </c>
       <c r="J91" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K91" t="b">
         <v>1</v>
@@ -7387,34 +7431,34 @@
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C92" t="s">
         <v>14</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E92" t="s">
         <v>145</v>
       </c>
       <c r="F92" t="s">
-        <v>316</v>
+        <v>447</v>
       </c>
       <c r="G92" t="s">
         <v>281</v>
       </c>
       <c r="H92" t="s">
-        <v>316</v>
+        <v>448</v>
       </c>
       <c r="I92" t="s">
         <v>19</v>
       </c>
       <c r="J92" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="K92" t="b">
         <v>1</v>
@@ -7431,34 +7475,34 @@
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C93" t="s">
         <v>14</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="E93" t="s">
         <v>145</v>
       </c>
       <c r="F93" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="G93" t="s">
         <v>281</v>
       </c>
       <c r="H93" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="I93" t="s">
         <v>19</v>
       </c>
       <c r="J93" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="K93" t="b">
         <v>1</v>
@@ -7475,34 +7519,34 @@
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C94" t="s">
         <v>14</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="E94" t="s">
         <v>145</v>
       </c>
       <c r="F94" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="G94" t="s">
         <v>281</v>
       </c>
       <c r="H94" t="s">
-        <v>446</v>
+        <v>566</v>
       </c>
       <c r="I94" t="s">
         <v>19</v>
       </c>
       <c r="J94" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="K94" t="b">
         <v>1</v>
@@ -7519,34 +7563,34 @@
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C95" t="s">
         <v>14</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E95" t="s">
         <v>145</v>
       </c>
       <c r="F95" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="G95" t="s">
         <v>281</v>
       </c>
       <c r="H95" t="s">
-        <v>566</v>
+        <v>444</v>
       </c>
       <c r="I95" t="s">
         <v>19</v>
       </c>
       <c r="J95" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="K95" t="b">
         <v>1</v>
@@ -7563,34 +7607,34 @@
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="C96" t="s">
         <v>14</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E96" t="s">
         <v>145</v>
       </c>
       <c r="F96" t="s">
-        <v>444</v>
+        <v>332</v>
       </c>
       <c r="G96" t="s">
         <v>281</v>
       </c>
       <c r="H96" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="I96" t="s">
         <v>19</v>
       </c>
       <c r="J96" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="K96" t="b">
         <v>1</v>
@@ -7607,34 +7651,34 @@
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="C97" t="s">
         <v>14</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E97" t="s">
         <v>145</v>
       </c>
       <c r="F97" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="G97" t="s">
         <v>281</v>
       </c>
       <c r="H97" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
       <c r="I97" t="s">
         <v>19</v>
       </c>
       <c r="J97" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="K97" t="b">
         <v>1</v>
@@ -7651,34 +7695,34 @@
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="C98" t="s">
         <v>14</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E98" t="s">
         <v>145</v>
       </c>
       <c r="F98" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="G98" t="s">
         <v>281</v>
       </c>
       <c r="H98" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="I98" t="s">
         <v>19</v>
       </c>
       <c r="J98" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="K98" t="b">
         <v>1</v>
@@ -7695,34 +7739,34 @@
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="C99" t="s">
         <v>14</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E99" t="s">
         <v>145</v>
       </c>
       <c r="F99" t="s">
-        <v>340</v>
+        <v>438</v>
       </c>
       <c r="G99" t="s">
         <v>281</v>
       </c>
       <c r="H99" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I99" t="s">
         <v>19</v>
       </c>
       <c r="J99" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="K99" t="b">
         <v>1</v>
@@ -7739,34 +7783,34 @@
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C100" t="s">
         <v>14</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E100" t="s">
         <v>145</v>
       </c>
       <c r="F100" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="G100" t="s">
         <v>281</v>
       </c>
       <c r="H100" t="s">
-        <v>441</v>
+        <v>347</v>
       </c>
       <c r="I100" t="s">
         <v>19</v>
       </c>
       <c r="J100" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="K100" t="b">
         <v>1</v>
@@ -7783,34 +7827,34 @@
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="C101" t="s">
         <v>14</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E101" t="s">
         <v>145</v>
       </c>
       <c r="F101" t="s">
-        <v>437</v>
+        <v>352</v>
       </c>
       <c r="G101" t="s">
         <v>281</v>
       </c>
       <c r="H101" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="I101" t="s">
         <v>19</v>
       </c>
       <c r="J101" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="K101" t="b">
         <v>1</v>
@@ -7825,52 +7869,8 @@
         <v>82</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A102" t="s">
-        <v>348</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>349</v>
-      </c>
-      <c r="C102" t="s">
-        <v>14</v>
-      </c>
-      <c r="D102" s="2" t="s">
-        <v>436</v>
-      </c>
-      <c r="E102" t="s">
-        <v>145</v>
-      </c>
-      <c r="F102" t="s">
-        <v>352</v>
-      </c>
-      <c r="G102" t="s">
-        <v>281</v>
-      </c>
-      <c r="H102" t="s">
-        <v>351</v>
-      </c>
-      <c r="I102" t="s">
-        <v>19</v>
-      </c>
-      <c r="J102" t="s">
-        <v>350</v>
-      </c>
-      <c r="K102" t="b">
-        <v>1</v>
-      </c>
-      <c r="L102" t="b">
-        <v>1</v>
-      </c>
-      <c r="M102">
-        <v>1</v>
-      </c>
-      <c r="N102">
-        <v>82</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N102" xr:uid="{D2038D1B-0BDF-4C41-81D3-AA444C04F44C}"/>
+  <autoFilter ref="A1:N101" xr:uid="{D2038D1B-0BDF-4C41-81D3-AA444C04F44C}"/>
   <phoneticPr fontId="18"/>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" xr:uid="{A2D0AE02-39E8-4AE3-8B46-936177CA49B7}"/>
@@ -7882,88 +7882,89 @@
     <hyperlink ref="D10" r:id="rId7" xr:uid="{5B8EE01A-5A13-4380-AC53-2390FD449498}"/>
     <hyperlink ref="D12" r:id="rId8" xr:uid="{0D612A1F-9385-4A87-899B-1B70D7E9F2FE}"/>
     <hyperlink ref="D15" r:id="rId9" xr:uid="{0F056084-D571-41F2-8ACC-A5D9DF095541}"/>
-    <hyperlink ref="D17" r:id="rId10" xr:uid="{4E2AB146-6CF3-4217-8C09-499F7C887D24}"/>
-    <hyperlink ref="D18" r:id="rId11" xr:uid="{164AC54B-ABE4-40B8-B65F-E7A73A55A4C4}"/>
-    <hyperlink ref="D19" r:id="rId12" xr:uid="{A898E907-8504-4478-AA23-6B9C1EC504B1}"/>
-    <hyperlink ref="D20" r:id="rId13" xr:uid="{68F9D4AB-A268-4402-AAD1-A0429050B044}"/>
-    <hyperlink ref="D21" r:id="rId14" xr:uid="{9C194E30-142D-432A-B1C7-AB3AE9CACF94}"/>
-    <hyperlink ref="D22" r:id="rId15" xr:uid="{5A570FA5-E5F5-49E3-8FF9-DBAC269CC05F}"/>
-    <hyperlink ref="D23" r:id="rId16" xr:uid="{C64FB3D3-B238-4C1C-8CB1-837BC2BCDE52}"/>
-    <hyperlink ref="D25" r:id="rId17" xr:uid="{0C5E4962-8414-43B1-9793-641C6EDEF909}"/>
-    <hyperlink ref="D26" r:id="rId18" xr:uid="{2B397B98-6863-44E2-8B37-593F469D113D}"/>
-    <hyperlink ref="D31" r:id="rId19" xr:uid="{5089B3EA-FBEC-4CF9-AC82-D6E795C2F3E6}"/>
-    <hyperlink ref="D32" r:id="rId20" xr:uid="{B1EC4A91-5D46-4385-B298-4FB7D680CC3D}"/>
-    <hyperlink ref="D33" r:id="rId21" xr:uid="{995E1367-FF74-4CE5-AB91-7770E2E033FB}"/>
-    <hyperlink ref="D34" r:id="rId22" xr:uid="{45D69CA8-71E1-4B5C-9C4F-1CCE59B93952}"/>
-    <hyperlink ref="D35" r:id="rId23" xr:uid="{C25CD590-E249-49B1-B1F1-499DAD8E0E86}"/>
-    <hyperlink ref="D36" r:id="rId24" xr:uid="{1AB1A130-5FE8-485A-8941-7C2143D41B06}"/>
-    <hyperlink ref="D37" r:id="rId25" xr:uid="{BA050A5D-CDE9-41FB-92A3-45739B6A1ED8}"/>
-    <hyperlink ref="D38" r:id="rId26" xr:uid="{5BAA0279-5263-455E-B2CC-DD1A8D3CFC04}"/>
-    <hyperlink ref="D39" r:id="rId27" xr:uid="{62D15C57-9EA1-48EA-A324-F006945BB4BB}"/>
-    <hyperlink ref="D40" r:id="rId28" xr:uid="{41BCE278-C575-4835-B0B8-91DF79D1FD4B}"/>
-    <hyperlink ref="D41" r:id="rId29" xr:uid="{4D237A78-9C43-4C8C-90A3-CDC5505AA0F6}"/>
-    <hyperlink ref="D43" r:id="rId30" xr:uid="{6D70EA67-1745-4AC3-8493-2F9F6125B93C}"/>
-    <hyperlink ref="D44" r:id="rId31" xr:uid="{3F3953EB-2581-4423-A728-000BF2493078}"/>
-    <hyperlink ref="D45" r:id="rId32" xr:uid="{BBED1518-2B7E-491A-83AE-8AB14F5D10DA}"/>
-    <hyperlink ref="D46" r:id="rId33" xr:uid="{ADDD5B8D-D5E7-47F8-9241-A1CC52332F43}"/>
-    <hyperlink ref="D48" r:id="rId34" xr:uid="{24188C79-265E-4185-B3B8-54F80F947ABC}"/>
-    <hyperlink ref="D49" r:id="rId35" xr:uid="{F478252C-BAB1-4886-8C2E-5D19C69C1E2A}"/>
-    <hyperlink ref="D50" r:id="rId36" xr:uid="{41CF7F1A-2E74-4CBB-8816-9644EB34711A}"/>
-    <hyperlink ref="D52" r:id="rId37" xr:uid="{8D079AB8-2D56-4A2D-BC11-F10816C096F8}"/>
-    <hyperlink ref="D54" r:id="rId38" xr:uid="{44DC06DE-25DB-4042-8D17-F624248C9741}"/>
-    <hyperlink ref="D55" r:id="rId39" xr:uid="{92578218-E9FE-4D00-A7D1-65831EB24769}"/>
-    <hyperlink ref="D56" r:id="rId40" xr:uid="{E664A7A6-9B89-42B9-8556-04DEE2C17A7B}"/>
-    <hyperlink ref="D57" r:id="rId41" xr:uid="{AD86BCE5-6742-4A1E-8C6B-9FCEBD57FE05}"/>
-    <hyperlink ref="D58" r:id="rId42" xr:uid="{F1325C0E-80C5-4747-ACFB-50AC1CF881EB}"/>
-    <hyperlink ref="D60" r:id="rId43" xr:uid="{757E03E7-87F1-4660-ADE2-863F74482037}"/>
-    <hyperlink ref="D61" r:id="rId44" xr:uid="{051FD699-7AC6-4215-8F95-BF066E4C5E80}"/>
-    <hyperlink ref="D62" r:id="rId45" xr:uid="{95F43FA4-0A4C-45BA-BF6B-AEF2E902E68F}"/>
-    <hyperlink ref="D63" r:id="rId46" xr:uid="{66BF6C8F-5B87-43E6-8D53-B9EEFCAD20FF}"/>
-    <hyperlink ref="D64" r:id="rId47" xr:uid="{C3B62239-CA47-4E47-97E7-C6EB3594ABEC}"/>
-    <hyperlink ref="D65" r:id="rId48" xr:uid="{FEF3E352-081C-4539-B8CB-D2004D8F850F}"/>
-    <hyperlink ref="D66" r:id="rId49" xr:uid="{BBA51556-F0D4-45FE-89D4-A2D808F3881D}"/>
-    <hyperlink ref="D67" r:id="rId50" xr:uid="{05B81A66-63EF-459B-9D35-7874264C6497}"/>
-    <hyperlink ref="D68" r:id="rId51" xr:uid="{A60053B2-6C0A-434F-9446-795B1AEAB31E}"/>
-    <hyperlink ref="D69" r:id="rId52" xr:uid="{68931F73-7867-4D77-AE35-552FB7DC72AD}"/>
-    <hyperlink ref="D70" r:id="rId53" xr:uid="{23FB3BE7-CDEC-4100-8C79-EF3853AD6CDE}"/>
-    <hyperlink ref="D71" r:id="rId54" xr:uid="{15A882FA-8FBF-4DE1-B229-CC158121D767}"/>
-    <hyperlink ref="D73" r:id="rId55" xr:uid="{F5547B44-44B0-4C60-922F-29470EC07569}"/>
-    <hyperlink ref="D74" r:id="rId56" xr:uid="{5A1E9648-41ED-492F-8DCF-0B2D5631D032}"/>
-    <hyperlink ref="D75" r:id="rId57" xr:uid="{8E925288-A601-44FC-BA3E-2B8CDCD6FD92}"/>
-    <hyperlink ref="D76" r:id="rId58" xr:uid="{FDDA423D-5ED7-4998-B9E8-7EBBC66BFD30}"/>
-    <hyperlink ref="D77" r:id="rId59" xr:uid="{BBAD925D-B448-4FAD-9D89-27E5C24CF992}"/>
-    <hyperlink ref="D78" r:id="rId60" xr:uid="{0873E3AB-F27C-49C9-A52B-70F216F7E335}"/>
-    <hyperlink ref="D79" r:id="rId61" xr:uid="{1587CF04-BB87-47C9-99D5-159BF52298B2}"/>
-    <hyperlink ref="D80" r:id="rId62" xr:uid="{5DBBC488-8A82-4465-937A-A05D644D7DA4}"/>
-    <hyperlink ref="D81" r:id="rId63" xr:uid="{0E6868DB-A2DC-4C3C-8369-6C90F47AA51D}"/>
-    <hyperlink ref="D82" r:id="rId64" xr:uid="{BCA2F466-1783-4194-A940-0BE51143B570}"/>
-    <hyperlink ref="D83" r:id="rId65" xr:uid="{04850A9C-5CFA-442B-BE92-B59D315F4A26}"/>
-    <hyperlink ref="D84" r:id="rId66" xr:uid="{919E18D4-0BE3-42EE-A227-FC2658E8A852}"/>
-    <hyperlink ref="D85" r:id="rId67" xr:uid="{2EC0B72D-B7AF-434B-80CB-89B6D7BCAABC}"/>
-    <hyperlink ref="D86" r:id="rId68" xr:uid="{F13612BA-DB02-4B0F-ACD8-8ACCE9CAA6CF}"/>
-    <hyperlink ref="D87" r:id="rId69" xr:uid="{506E9E49-B52A-4D63-9357-86C27EB89419}"/>
-    <hyperlink ref="D88" r:id="rId70" xr:uid="{4534AEFB-C2DC-4B8C-9E21-FF7B8DC3B517}"/>
-    <hyperlink ref="D89" r:id="rId71" xr:uid="{0775E04B-01BD-47A3-ADC5-DB292F5CC258}"/>
-    <hyperlink ref="D90" r:id="rId72" xr:uid="{AD1C2331-74A0-4340-A639-1CE48438E20B}"/>
-    <hyperlink ref="D91" r:id="rId73" xr:uid="{99F7FE63-2CD9-48B5-97A0-7745574E29A3}"/>
-    <hyperlink ref="D92" r:id="rId74" xr:uid="{7F81C9DB-B62F-4DC3-9EC1-761C73DE97DD}"/>
-    <hyperlink ref="D93" r:id="rId75" xr:uid="{38FE4A68-681E-43EC-9940-DF9D7A126DE3}"/>
-    <hyperlink ref="D94" r:id="rId76" xr:uid="{4BD9B3F4-D16A-479F-B8EF-E7AE1FA56031}"/>
-    <hyperlink ref="D95" r:id="rId77" xr:uid="{FC43E27C-35EC-4168-B499-783A6E8602ED}"/>
-    <hyperlink ref="D96" r:id="rId78" xr:uid="{0A310316-F2CF-49CD-8070-73B82ECD308A}"/>
-    <hyperlink ref="D97" r:id="rId79" xr:uid="{498A75A1-FCF2-4BDD-9F2E-F2BF24297229}"/>
-    <hyperlink ref="D98" r:id="rId80" xr:uid="{4CD9DC76-9471-4820-B7AF-4F91E714ECFD}"/>
-    <hyperlink ref="D99" r:id="rId81" xr:uid="{5A1BAE36-4FAC-4DC4-9692-ED100AFB5243}"/>
-    <hyperlink ref="D100" r:id="rId82" xr:uid="{D0C2DA9B-7FA7-4CE8-ABA2-6E4AD7A4FA3B}"/>
-    <hyperlink ref="D101" r:id="rId83" xr:uid="{04BE2678-F9CE-4C22-B8C2-AE50369C7A51}"/>
-    <hyperlink ref="D102" r:id="rId84" xr:uid="{86B8B830-57AA-4373-B839-6E939275BF77}"/>
+    <hyperlink ref="D16" r:id="rId10" xr:uid="{4E2AB146-6CF3-4217-8C09-499F7C887D24}"/>
+    <hyperlink ref="D17" r:id="rId11" xr:uid="{164AC54B-ABE4-40B8-B65F-E7A73A55A4C4}"/>
+    <hyperlink ref="D18" r:id="rId12" xr:uid="{A898E907-8504-4478-AA23-6B9C1EC504B1}"/>
+    <hyperlink ref="D19" r:id="rId13" xr:uid="{68F9D4AB-A268-4402-AAD1-A0429050B044}"/>
+    <hyperlink ref="D20" r:id="rId14" xr:uid="{9C194E30-142D-432A-B1C7-AB3AE9CACF94}"/>
+    <hyperlink ref="D21" r:id="rId15" xr:uid="{5A570FA5-E5F5-49E3-8FF9-DBAC269CC05F}"/>
+    <hyperlink ref="D22" r:id="rId16" xr:uid="{C64FB3D3-B238-4C1C-8CB1-837BC2BCDE52}"/>
+    <hyperlink ref="D24" r:id="rId17" xr:uid="{0C5E4962-8414-43B1-9793-641C6EDEF909}"/>
+    <hyperlink ref="D25" r:id="rId18" xr:uid="{2B397B98-6863-44E2-8B37-593F469D113D}"/>
+    <hyperlink ref="D30" r:id="rId19" xr:uid="{5089B3EA-FBEC-4CF9-AC82-D6E795C2F3E6}"/>
+    <hyperlink ref="D31" r:id="rId20" xr:uid="{B1EC4A91-5D46-4385-B298-4FB7D680CC3D}"/>
+    <hyperlink ref="D32" r:id="rId21" xr:uid="{995E1367-FF74-4CE5-AB91-7770E2E033FB}"/>
+    <hyperlink ref="D33" r:id="rId22" xr:uid="{45D69CA8-71E1-4B5C-9C4F-1CCE59B93952}"/>
+    <hyperlink ref="D34" r:id="rId23" xr:uid="{C25CD590-E249-49B1-B1F1-499DAD8E0E86}"/>
+    <hyperlink ref="D35" r:id="rId24" xr:uid="{1AB1A130-5FE8-485A-8941-7C2143D41B06}"/>
+    <hyperlink ref="D36" r:id="rId25" xr:uid="{BA050A5D-CDE9-41FB-92A3-45739B6A1ED8}"/>
+    <hyperlink ref="D37" r:id="rId26" xr:uid="{5BAA0279-5263-455E-B2CC-DD1A8D3CFC04}"/>
+    <hyperlink ref="D38" r:id="rId27" xr:uid="{62D15C57-9EA1-48EA-A324-F006945BB4BB}"/>
+    <hyperlink ref="D39" r:id="rId28" xr:uid="{41BCE278-C575-4835-B0B8-91DF79D1FD4B}"/>
+    <hyperlink ref="D40" r:id="rId29" xr:uid="{4D237A78-9C43-4C8C-90A3-CDC5505AA0F6}"/>
+    <hyperlink ref="D42" r:id="rId30" xr:uid="{6D70EA67-1745-4AC3-8493-2F9F6125B93C}"/>
+    <hyperlink ref="D43" r:id="rId31" xr:uid="{3F3953EB-2581-4423-A728-000BF2493078}"/>
+    <hyperlink ref="D44" r:id="rId32" xr:uid="{BBED1518-2B7E-491A-83AE-8AB14F5D10DA}"/>
+    <hyperlink ref="D45" r:id="rId33" xr:uid="{ADDD5B8D-D5E7-47F8-9241-A1CC52332F43}"/>
+    <hyperlink ref="D47" r:id="rId34" xr:uid="{24188C79-265E-4185-B3B8-54F80F947ABC}"/>
+    <hyperlink ref="D48" r:id="rId35" xr:uid="{F478252C-BAB1-4886-8C2E-5D19C69C1E2A}"/>
+    <hyperlink ref="D49" r:id="rId36" xr:uid="{41CF7F1A-2E74-4CBB-8816-9644EB34711A}"/>
+    <hyperlink ref="D51" r:id="rId37" xr:uid="{8D079AB8-2D56-4A2D-BC11-F10816C096F8}"/>
+    <hyperlink ref="D53" r:id="rId38" xr:uid="{44DC06DE-25DB-4042-8D17-F624248C9741}"/>
+    <hyperlink ref="D54" r:id="rId39" xr:uid="{92578218-E9FE-4D00-A7D1-65831EB24769}"/>
+    <hyperlink ref="D55" r:id="rId40" xr:uid="{E664A7A6-9B89-42B9-8556-04DEE2C17A7B}"/>
+    <hyperlink ref="D56" r:id="rId41" xr:uid="{AD86BCE5-6742-4A1E-8C6B-9FCEBD57FE05}"/>
+    <hyperlink ref="D57" r:id="rId42" xr:uid="{F1325C0E-80C5-4747-ACFB-50AC1CF881EB}"/>
+    <hyperlink ref="D59" r:id="rId43" xr:uid="{757E03E7-87F1-4660-ADE2-863F74482037}"/>
+    <hyperlink ref="D60" r:id="rId44" xr:uid="{051FD699-7AC6-4215-8F95-BF066E4C5E80}"/>
+    <hyperlink ref="D61" r:id="rId45" xr:uid="{95F43FA4-0A4C-45BA-BF6B-AEF2E902E68F}"/>
+    <hyperlink ref="D62" r:id="rId46" xr:uid="{66BF6C8F-5B87-43E6-8D53-B9EEFCAD20FF}"/>
+    <hyperlink ref="D63" r:id="rId47" xr:uid="{C3B62239-CA47-4E47-97E7-C6EB3594ABEC}"/>
+    <hyperlink ref="D64" r:id="rId48" xr:uid="{FEF3E352-081C-4539-B8CB-D2004D8F850F}"/>
+    <hyperlink ref="D65" r:id="rId49" xr:uid="{BBA51556-F0D4-45FE-89D4-A2D808F3881D}"/>
+    <hyperlink ref="D66" r:id="rId50" xr:uid="{05B81A66-63EF-459B-9D35-7874264C6497}"/>
+    <hyperlink ref="D67" r:id="rId51" xr:uid="{A60053B2-6C0A-434F-9446-795B1AEAB31E}"/>
+    <hyperlink ref="D68" r:id="rId52" xr:uid="{68931F73-7867-4D77-AE35-552FB7DC72AD}"/>
+    <hyperlink ref="D69" r:id="rId53" xr:uid="{23FB3BE7-CDEC-4100-8C79-EF3853AD6CDE}"/>
+    <hyperlink ref="D70" r:id="rId54" xr:uid="{15A882FA-8FBF-4DE1-B229-CC158121D767}"/>
+    <hyperlink ref="D72" r:id="rId55" xr:uid="{F5547B44-44B0-4C60-922F-29470EC07569}"/>
+    <hyperlink ref="D73" r:id="rId56" xr:uid="{5A1E9648-41ED-492F-8DCF-0B2D5631D032}"/>
+    <hyperlink ref="D74" r:id="rId57" xr:uid="{8E925288-A601-44FC-BA3E-2B8CDCD6FD92}"/>
+    <hyperlink ref="D75" r:id="rId58" xr:uid="{FDDA423D-5ED7-4998-B9E8-7EBBC66BFD30}"/>
+    <hyperlink ref="D76" r:id="rId59" xr:uid="{BBAD925D-B448-4FAD-9D89-27E5C24CF992}"/>
+    <hyperlink ref="D77" r:id="rId60" xr:uid="{0873E3AB-F27C-49C9-A52B-70F216F7E335}"/>
+    <hyperlink ref="D78" r:id="rId61" xr:uid="{1587CF04-BB87-47C9-99D5-159BF52298B2}"/>
+    <hyperlink ref="D79" r:id="rId62" xr:uid="{5DBBC488-8A82-4465-937A-A05D644D7DA4}"/>
+    <hyperlink ref="D80" r:id="rId63" xr:uid="{0E6868DB-A2DC-4C3C-8369-6C90F47AA51D}"/>
+    <hyperlink ref="D81" r:id="rId64" xr:uid="{BCA2F466-1783-4194-A940-0BE51143B570}"/>
+    <hyperlink ref="D82" r:id="rId65" xr:uid="{04850A9C-5CFA-442B-BE92-B59D315F4A26}"/>
+    <hyperlink ref="D83" r:id="rId66" xr:uid="{919E18D4-0BE3-42EE-A227-FC2658E8A852}"/>
+    <hyperlink ref="D84" r:id="rId67" xr:uid="{2EC0B72D-B7AF-434B-80CB-89B6D7BCAABC}"/>
+    <hyperlink ref="D85" r:id="rId68" xr:uid="{F13612BA-DB02-4B0F-ACD8-8ACCE9CAA6CF}"/>
+    <hyperlink ref="D86" r:id="rId69" xr:uid="{506E9E49-B52A-4D63-9357-86C27EB89419}"/>
+    <hyperlink ref="D87" r:id="rId70" xr:uid="{4534AEFB-C2DC-4B8C-9E21-FF7B8DC3B517}"/>
+    <hyperlink ref="D88" r:id="rId71" xr:uid="{0775E04B-01BD-47A3-ADC5-DB292F5CC258}"/>
+    <hyperlink ref="D89" r:id="rId72" xr:uid="{AD1C2331-74A0-4340-A639-1CE48438E20B}"/>
+    <hyperlink ref="D90" r:id="rId73" xr:uid="{99F7FE63-2CD9-48B5-97A0-7745574E29A3}"/>
+    <hyperlink ref="D91" r:id="rId74" xr:uid="{7F81C9DB-B62F-4DC3-9EC1-761C73DE97DD}"/>
+    <hyperlink ref="D92" r:id="rId75" xr:uid="{38FE4A68-681E-43EC-9940-DF9D7A126DE3}"/>
+    <hyperlink ref="D93" r:id="rId76" xr:uid="{4BD9B3F4-D16A-479F-B8EF-E7AE1FA56031}"/>
+    <hyperlink ref="D94" r:id="rId77" xr:uid="{FC43E27C-35EC-4168-B499-783A6E8602ED}"/>
+    <hyperlink ref="D95" r:id="rId78" xr:uid="{0A310316-F2CF-49CD-8070-73B82ECD308A}"/>
+    <hyperlink ref="D96" r:id="rId79" xr:uid="{498A75A1-FCF2-4BDD-9F2E-F2BF24297229}"/>
+    <hyperlink ref="D97" r:id="rId80" xr:uid="{4CD9DC76-9471-4820-B7AF-4F91E714ECFD}"/>
+    <hyperlink ref="D98" r:id="rId81" xr:uid="{5A1BAE36-4FAC-4DC4-9692-ED100AFB5243}"/>
+    <hyperlink ref="D99" r:id="rId82" xr:uid="{D0C2DA9B-7FA7-4CE8-ABA2-6E4AD7A4FA3B}"/>
+    <hyperlink ref="D100" r:id="rId83" xr:uid="{04BE2678-F9CE-4C22-B8C2-AE50369C7A51}"/>
+    <hyperlink ref="D101" r:id="rId84" xr:uid="{86B8B830-57AA-4373-B839-6E939275BF77}"/>
     <hyperlink ref="D13" r:id="rId85" xr:uid="{8D644E0F-AE8B-49CA-BCB1-CDA872D18BB6}"/>
     <hyperlink ref="D14" r:id="rId86" xr:uid="{AF6718EC-E480-4305-8568-A58DA187FD87}"/>
-    <hyperlink ref="D72" r:id="rId87" xr:uid="{5F8641B6-6F17-4D16-93FF-5EB87D0FDB14}"/>
-    <hyperlink ref="D47" r:id="rId88" xr:uid="{E2053B46-5E95-47CE-855E-9B0D90F9DE58}"/>
-    <hyperlink ref="D51" r:id="rId89" xr:uid="{08299D7B-C3E3-4DEF-940F-0CB8A95C2EAE}"/>
-    <hyperlink ref="D53" r:id="rId90" xr:uid="{9B2BA5D7-D300-445E-92E8-70B775A76017}"/>
-    <hyperlink ref="D59" r:id="rId91" xr:uid="{7F44AE8F-5E10-4A9E-B2D3-1A1B1A3D70F6}"/>
+    <hyperlink ref="D71" r:id="rId87" xr:uid="{5F8641B6-6F17-4D16-93FF-5EB87D0FDB14}"/>
+    <hyperlink ref="D46" r:id="rId88" xr:uid="{E2053B46-5E95-47CE-855E-9B0D90F9DE58}"/>
+    <hyperlink ref="D50" r:id="rId89" xr:uid="{08299D7B-C3E3-4DEF-940F-0CB8A95C2EAE}"/>
+    <hyperlink ref="D52" r:id="rId90" xr:uid="{9B2BA5D7-D300-445E-92E8-70B775A76017}"/>
+    <hyperlink ref="D58" r:id="rId91" xr:uid="{7F44AE8F-5E10-4A9E-B2D3-1A1B1A3D70F6}"/>
+    <hyperlink ref="D41" r:id="rId92" xr:uid="{9D7FB1F9-1541-4520-BB0C-141B6F8B9160}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>